<commit_message>
Add intake drop-folder auto-import to the 15-min job
Team members fill the template offline and drop it in an 'Intake Inbox'
folder; the schedule imports it for them.

- Import-Intake.ps1: scans Intake Inbox, appends 'Enter Here' rows A-L into
  the master 'Project Tasks' via Excel COM (lossless - charts/tables/Gantt
  preserved), archives processed files, rejects non-intake files. Only wakes
  Excel when files are waiting; bails safely if the master is open.
- Update-Auto.ps1: runs the import first, then export + Azure push, so new
  rows reach the dashboard the same cycle. Import errors never block export.
- Template: Start/Finish pre-formatted as dates so typed values parse; tip
  now points users to the Intake Inbox folder.
- INTAKE-AUTOIMPORT.md: setup + runbook + troubleshooting.

https://claude.ai/code/session_01WJTcYohvXPdyiEYiaxvXwj
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -61,11 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -432,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -517,6 +520,8 @@
           <t>Phase 1 - Planning</t>
         </is>
       </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -527,9 +532,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Tip: pick your Project (A), then fill Task, Start/Finish dates and Assigned for each phase. Add rows as needed; delete phases you don't use. Save and send back — it gets imported into the master schedule.</t>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Tip: pick your Project (A), then fill Task, Start/Finish dates and Assigned for each phase. Add rows as needed; delete phases you don't use. When done, save this file and drop it in the team 'Intake Inbox' folder (ask your PM for the link) — it imports into the schedule automatically. Use real dates in Start/Finish (e.g. 6/15/26).</t>
         </is>
       </c>
     </row>
@@ -539,6 +544,8 @@
           <t>Phase 2 - Design &amp; Detail</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -556,6 +563,8 @@
           <t>Phase 3 - Fabrication</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -573,6 +582,8 @@
           <t>Phase 4 - Electrical &amp; Technology Integration</t>
         </is>
       </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -590,6 +601,8 @@
           <t>Phase 5 - Graphics, Soft Launch / QS / Handover</t>
         </is>
       </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -600,6 +613,1182 @@
           <t>No</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="E98" s="2" t="n"/>
+      <c r="F98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="E102" s="2" t="n"/>
+      <c r="F102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="E104" s="2" t="n"/>
+      <c r="F104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="E105" s="2" t="n"/>
+      <c r="F105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="E106" s="2" t="n"/>
+      <c r="F106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="E107" s="2" t="n"/>
+      <c r="F107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="E109" s="2" t="n"/>
+      <c r="F109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="E112" s="2" t="n"/>
+      <c r="F112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="E113" s="2" t="n"/>
+      <c r="F113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="E114" s="2" t="n"/>
+      <c r="F114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="E115" s="2" t="n"/>
+      <c r="F115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="E116" s="2" t="n"/>
+      <c r="F116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="E117" s="2" t="n"/>
+      <c r="F117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="E118" s="2" t="n"/>
+      <c r="F118" s="2" t="n"/>
+    </row>
+    <row r="119">
+      <c r="E119" s="2" t="n"/>
+      <c r="F119" s="2" t="n"/>
+    </row>
+    <row r="120">
+      <c r="E120" s="2" t="n"/>
+      <c r="F120" s="2" t="n"/>
+    </row>
+    <row r="121">
+      <c r="E121" s="2" t="n"/>
+      <c r="F121" s="2" t="n"/>
+    </row>
+    <row r="122">
+      <c r="E122" s="2" t="n"/>
+      <c r="F122" s="2" t="n"/>
+    </row>
+    <row r="123">
+      <c r="E123" s="2" t="n"/>
+      <c r="F123" s="2" t="n"/>
+    </row>
+    <row r="124">
+      <c r="E124" s="2" t="n"/>
+      <c r="F124" s="2" t="n"/>
+    </row>
+    <row r="125">
+      <c r="E125" s="2" t="n"/>
+      <c r="F125" s="2" t="n"/>
+    </row>
+    <row r="126">
+      <c r="E126" s="2" t="n"/>
+      <c r="F126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="E127" s="2" t="n"/>
+      <c r="F127" s="2" t="n"/>
+    </row>
+    <row r="128">
+      <c r="E128" s="2" t="n"/>
+      <c r="F128" s="2" t="n"/>
+    </row>
+    <row r="129">
+      <c r="E129" s="2" t="n"/>
+      <c r="F129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="E130" s="2" t="n"/>
+      <c r="F130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="E131" s="2" t="n"/>
+      <c r="F131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="E132" s="2" t="n"/>
+      <c r="F132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="E133" s="2" t="n"/>
+      <c r="F133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="E134" s="2" t="n"/>
+      <c r="F134" s="2" t="n"/>
+    </row>
+    <row r="135">
+      <c r="E135" s="2" t="n"/>
+      <c r="F135" s="2" t="n"/>
+    </row>
+    <row r="136">
+      <c r="E136" s="2" t="n"/>
+      <c r="F136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="E137" s="2" t="n"/>
+      <c r="F137" s="2" t="n"/>
+    </row>
+    <row r="138">
+      <c r="E138" s="2" t="n"/>
+      <c r="F138" s="2" t="n"/>
+    </row>
+    <row r="139">
+      <c r="E139" s="2" t="n"/>
+      <c r="F139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="E140" s="2" t="n"/>
+      <c r="F140" s="2" t="n"/>
+    </row>
+    <row r="141">
+      <c r="E141" s="2" t="n"/>
+      <c r="F141" s="2" t="n"/>
+    </row>
+    <row r="142">
+      <c r="E142" s="2" t="n"/>
+      <c r="F142" s="2" t="n"/>
+    </row>
+    <row r="143">
+      <c r="E143" s="2" t="n"/>
+      <c r="F143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="E144" s="2" t="n"/>
+      <c r="F144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="E145" s="2" t="n"/>
+      <c r="F145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="E146" s="2" t="n"/>
+      <c r="F146" s="2" t="n"/>
+    </row>
+    <row r="147">
+      <c r="E147" s="2" t="n"/>
+      <c r="F147" s="2" t="n"/>
+    </row>
+    <row r="148">
+      <c r="E148" s="2" t="n"/>
+      <c r="F148" s="2" t="n"/>
+    </row>
+    <row r="149">
+      <c r="E149" s="2" t="n"/>
+      <c r="F149" s="2" t="n"/>
+    </row>
+    <row r="150">
+      <c r="E150" s="2" t="n"/>
+      <c r="F150" s="2" t="n"/>
+    </row>
+    <row r="151">
+      <c r="E151" s="2" t="n"/>
+      <c r="F151" s="2" t="n"/>
+    </row>
+    <row r="152">
+      <c r="E152" s="2" t="n"/>
+      <c r="F152" s="2" t="n"/>
+    </row>
+    <row r="153">
+      <c r="E153" s="2" t="n"/>
+      <c r="F153" s="2" t="n"/>
+    </row>
+    <row r="154">
+      <c r="E154" s="2" t="n"/>
+      <c r="F154" s="2" t="n"/>
+    </row>
+    <row r="155">
+      <c r="E155" s="2" t="n"/>
+      <c r="F155" s="2" t="n"/>
+    </row>
+    <row r="156">
+      <c r="E156" s="2" t="n"/>
+      <c r="F156" s="2" t="n"/>
+    </row>
+    <row r="157">
+      <c r="E157" s="2" t="n"/>
+      <c r="F157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="E158" s="2" t="n"/>
+      <c r="F158" s="2" t="n"/>
+    </row>
+    <row r="159">
+      <c r="E159" s="2" t="n"/>
+      <c r="F159" s="2" t="n"/>
+    </row>
+    <row r="160">
+      <c r="E160" s="2" t="n"/>
+      <c r="F160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="E161" s="2" t="n"/>
+      <c r="F161" s="2" t="n"/>
+    </row>
+    <row r="162">
+      <c r="E162" s="2" t="n"/>
+      <c r="F162" s="2" t="n"/>
+    </row>
+    <row r="163">
+      <c r="E163" s="2" t="n"/>
+      <c r="F163" s="2" t="n"/>
+    </row>
+    <row r="164">
+      <c r="E164" s="2" t="n"/>
+      <c r="F164" s="2" t="n"/>
+    </row>
+    <row r="165">
+      <c r="E165" s="2" t="n"/>
+      <c r="F165" s="2" t="n"/>
+    </row>
+    <row r="166">
+      <c r="E166" s="2" t="n"/>
+      <c r="F166" s="2" t="n"/>
+    </row>
+    <row r="167">
+      <c r="E167" s="2" t="n"/>
+      <c r="F167" s="2" t="n"/>
+    </row>
+    <row r="168">
+      <c r="E168" s="2" t="n"/>
+      <c r="F168" s="2" t="n"/>
+    </row>
+    <row r="169">
+      <c r="E169" s="2" t="n"/>
+      <c r="F169" s="2" t="n"/>
+    </row>
+    <row r="170">
+      <c r="E170" s="2" t="n"/>
+      <c r="F170" s="2" t="n"/>
+    </row>
+    <row r="171">
+      <c r="E171" s="2" t="n"/>
+      <c r="F171" s="2" t="n"/>
+    </row>
+    <row r="172">
+      <c r="E172" s="2" t="n"/>
+      <c r="F172" s="2" t="n"/>
+    </row>
+    <row r="173">
+      <c r="E173" s="2" t="n"/>
+      <c r="F173" s="2" t="n"/>
+    </row>
+    <row r="174">
+      <c r="E174" s="2" t="n"/>
+      <c r="F174" s="2" t="n"/>
+    </row>
+    <row r="175">
+      <c r="E175" s="2" t="n"/>
+      <c r="F175" s="2" t="n"/>
+    </row>
+    <row r="176">
+      <c r="E176" s="2" t="n"/>
+      <c r="F176" s="2" t="n"/>
+    </row>
+    <row r="177">
+      <c r="E177" s="2" t="n"/>
+      <c r="F177" s="2" t="n"/>
+    </row>
+    <row r="178">
+      <c r="E178" s="2" t="n"/>
+      <c r="F178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="E179" s="2" t="n"/>
+      <c r="F179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="E180" s="2" t="n"/>
+      <c r="F180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="E181" s="2" t="n"/>
+      <c r="F181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="E182" s="2" t="n"/>
+      <c r="F182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="E183" s="2" t="n"/>
+      <c r="F183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="E184" s="2" t="n"/>
+      <c r="F184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="E185" s="2" t="n"/>
+      <c r="F185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="E186" s="2" t="n"/>
+      <c r="F186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="E187" s="2" t="n"/>
+      <c r="F187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="E188" s="2" t="n"/>
+      <c r="F188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="E189" s="2" t="n"/>
+      <c r="F189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="E190" s="2" t="n"/>
+      <c r="F190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="E191" s="2" t="n"/>
+      <c r="F191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="E192" s="2" t="n"/>
+      <c r="F192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="E193" s="2" t="n"/>
+      <c r="F193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="E194" s="2" t="n"/>
+      <c r="F194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="E195" s="2" t="n"/>
+      <c r="F195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="E196" s="2" t="n"/>
+      <c r="F196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="E197" s="2" t="n"/>
+      <c r="F197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="E198" s="2" t="n"/>
+      <c r="F198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="E199" s="2" t="n"/>
+      <c r="F199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="E200" s="2" t="n"/>
+      <c r="F200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="E201" s="2" t="n"/>
+      <c r="F201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="E202" s="2" t="n"/>
+      <c r="F202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="E203" s="2" t="n"/>
+      <c r="F203" s="2" t="n"/>
+    </row>
+    <row r="204">
+      <c r="E204" s="2" t="n"/>
+      <c r="F204" s="2" t="n"/>
+    </row>
+    <row r="205">
+      <c r="E205" s="2" t="n"/>
+      <c r="F205" s="2" t="n"/>
+    </row>
+    <row r="206">
+      <c r="E206" s="2" t="n"/>
+      <c r="F206" s="2" t="n"/>
+    </row>
+    <row r="207">
+      <c r="E207" s="2" t="n"/>
+      <c r="F207" s="2" t="n"/>
+    </row>
+    <row r="208">
+      <c r="E208" s="2" t="n"/>
+      <c r="F208" s="2" t="n"/>
+    </row>
+    <row r="209">
+      <c r="E209" s="2" t="n"/>
+      <c r="F209" s="2" t="n"/>
+    </row>
+    <row r="210">
+      <c r="E210" s="2" t="n"/>
+      <c r="F210" s="2" t="n"/>
+    </row>
+    <row r="211">
+      <c r="E211" s="2" t="n"/>
+      <c r="F211" s="2" t="n"/>
+    </row>
+    <row r="212">
+      <c r="E212" s="2" t="n"/>
+      <c r="F212" s="2" t="n"/>
+    </row>
+    <row r="213">
+      <c r="E213" s="2" t="n"/>
+      <c r="F213" s="2" t="n"/>
+    </row>
+    <row r="214">
+      <c r="E214" s="2" t="n"/>
+      <c r="F214" s="2" t="n"/>
+    </row>
+    <row r="215">
+      <c r="E215" s="2" t="n"/>
+      <c r="F215" s="2" t="n"/>
+    </row>
+    <row r="216">
+      <c r="E216" s="2" t="n"/>
+      <c r="F216" s="2" t="n"/>
+    </row>
+    <row r="217">
+      <c r="E217" s="2" t="n"/>
+      <c r="F217" s="2" t="n"/>
+    </row>
+    <row r="218">
+      <c r="E218" s="2" t="n"/>
+      <c r="F218" s="2" t="n"/>
+    </row>
+    <row r="219">
+      <c r="E219" s="2" t="n"/>
+      <c r="F219" s="2" t="n"/>
+    </row>
+    <row r="220">
+      <c r="E220" s="2" t="n"/>
+      <c r="F220" s="2" t="n"/>
+    </row>
+    <row r="221">
+      <c r="E221" s="2" t="n"/>
+      <c r="F221" s="2" t="n"/>
+    </row>
+    <row r="222">
+      <c r="E222" s="2" t="n"/>
+      <c r="F222" s="2" t="n"/>
+    </row>
+    <row r="223">
+      <c r="E223" s="2" t="n"/>
+      <c r="F223" s="2" t="n"/>
+    </row>
+    <row r="224">
+      <c r="E224" s="2" t="n"/>
+      <c r="F224" s="2" t="n"/>
+    </row>
+    <row r="225">
+      <c r="E225" s="2" t="n"/>
+      <c r="F225" s="2" t="n"/>
+    </row>
+    <row r="226">
+      <c r="E226" s="2" t="n"/>
+      <c r="F226" s="2" t="n"/>
+    </row>
+    <row r="227">
+      <c r="E227" s="2" t="n"/>
+      <c r="F227" s="2" t="n"/>
+    </row>
+    <row r="228">
+      <c r="E228" s="2" t="n"/>
+      <c r="F228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="E229" s="2" t="n"/>
+      <c r="F229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="E230" s="2" t="n"/>
+      <c r="F230" s="2" t="n"/>
+    </row>
+    <row r="231">
+      <c r="E231" s="2" t="n"/>
+      <c r="F231" s="2" t="n"/>
+    </row>
+    <row r="232">
+      <c r="E232" s="2" t="n"/>
+      <c r="F232" s="2" t="n"/>
+    </row>
+    <row r="233">
+      <c r="E233" s="2" t="n"/>
+      <c r="F233" s="2" t="n"/>
+    </row>
+    <row r="234">
+      <c r="E234" s="2" t="n"/>
+      <c r="F234" s="2" t="n"/>
+    </row>
+    <row r="235">
+      <c r="E235" s="2" t="n"/>
+      <c r="F235" s="2" t="n"/>
+    </row>
+    <row r="236">
+      <c r="E236" s="2" t="n"/>
+      <c r="F236" s="2" t="n"/>
+    </row>
+    <row r="237">
+      <c r="E237" s="2" t="n"/>
+      <c r="F237" s="2" t="n"/>
+    </row>
+    <row r="238">
+      <c r="E238" s="2" t="n"/>
+      <c r="F238" s="2" t="n"/>
+    </row>
+    <row r="239">
+      <c r="E239" s="2" t="n"/>
+      <c r="F239" s="2" t="n"/>
+    </row>
+    <row r="240">
+      <c r="E240" s="2" t="n"/>
+      <c r="F240" s="2" t="n"/>
+    </row>
+    <row r="241">
+      <c r="E241" s="2" t="n"/>
+      <c r="F241" s="2" t="n"/>
+    </row>
+    <row r="242">
+      <c r="E242" s="2" t="n"/>
+      <c r="F242" s="2" t="n"/>
+    </row>
+    <row r="243">
+      <c r="E243" s="2" t="n"/>
+      <c r="F243" s="2" t="n"/>
+    </row>
+    <row r="244">
+      <c r="E244" s="2" t="n"/>
+      <c r="F244" s="2" t="n"/>
+    </row>
+    <row r="245">
+      <c r="E245" s="2" t="n"/>
+      <c r="F245" s="2" t="n"/>
+    </row>
+    <row r="246">
+      <c r="E246" s="2" t="n"/>
+      <c r="F246" s="2" t="n"/>
+    </row>
+    <row r="247">
+      <c r="E247" s="2" t="n"/>
+      <c r="F247" s="2" t="n"/>
+    </row>
+    <row r="248">
+      <c r="E248" s="2" t="n"/>
+      <c r="F248" s="2" t="n"/>
+    </row>
+    <row r="249">
+      <c r="E249" s="2" t="n"/>
+      <c r="F249" s="2" t="n"/>
+    </row>
+    <row r="250">
+      <c r="E250" s="2" t="n"/>
+      <c r="F250" s="2" t="n"/>
+    </row>
+    <row r="251">
+      <c r="E251" s="2" t="n"/>
+      <c r="F251" s="2" t="n"/>
+    </row>
+    <row r="252">
+      <c r="E252" s="2" t="n"/>
+      <c r="F252" s="2" t="n"/>
+    </row>
+    <row r="253">
+      <c r="E253" s="2" t="n"/>
+      <c r="F253" s="2" t="n"/>
+    </row>
+    <row r="254">
+      <c r="E254" s="2" t="n"/>
+      <c r="F254" s="2" t="n"/>
+    </row>
+    <row r="255">
+      <c r="E255" s="2" t="n"/>
+      <c r="F255" s="2" t="n"/>
+    </row>
+    <row r="256">
+      <c r="E256" s="2" t="n"/>
+      <c r="F256" s="2" t="n"/>
+    </row>
+    <row r="257">
+      <c r="E257" s="2" t="n"/>
+      <c r="F257" s="2" t="n"/>
+    </row>
+    <row r="258">
+      <c r="E258" s="2" t="n"/>
+      <c r="F258" s="2" t="n"/>
+    </row>
+    <row r="259">
+      <c r="E259" s="2" t="n"/>
+      <c r="F259" s="2" t="n"/>
+    </row>
+    <row r="260">
+      <c r="E260" s="2" t="n"/>
+      <c r="F260" s="2" t="n"/>
+    </row>
+    <row r="261">
+      <c r="E261" s="2" t="n"/>
+      <c r="F261" s="2" t="n"/>
+    </row>
+    <row r="262">
+      <c r="E262" s="2" t="n"/>
+      <c r="F262" s="2" t="n"/>
+    </row>
+    <row r="263">
+      <c r="E263" s="2" t="n"/>
+      <c r="F263" s="2" t="n"/>
+    </row>
+    <row r="264">
+      <c r="E264" s="2" t="n"/>
+      <c r="F264" s="2" t="n"/>
+    </row>
+    <row r="265">
+      <c r="E265" s="2" t="n"/>
+      <c r="F265" s="2" t="n"/>
+    </row>
+    <row r="266">
+      <c r="E266" s="2" t="n"/>
+      <c r="F266" s="2" t="n"/>
+    </row>
+    <row r="267">
+      <c r="E267" s="2" t="n"/>
+      <c r="F267" s="2" t="n"/>
+    </row>
+    <row r="268">
+      <c r="E268" s="2" t="n"/>
+      <c r="F268" s="2" t="n"/>
+    </row>
+    <row r="269">
+      <c r="E269" s="2" t="n"/>
+      <c r="F269" s="2" t="n"/>
+    </row>
+    <row r="270">
+      <c r="E270" s="2" t="n"/>
+      <c r="F270" s="2" t="n"/>
+    </row>
+    <row r="271">
+      <c r="E271" s="2" t="n"/>
+      <c r="F271" s="2" t="n"/>
+    </row>
+    <row r="272">
+      <c r="E272" s="2" t="n"/>
+      <c r="F272" s="2" t="n"/>
+    </row>
+    <row r="273">
+      <c r="E273" s="2" t="n"/>
+      <c r="F273" s="2" t="n"/>
+    </row>
+    <row r="274">
+      <c r="E274" s="2" t="n"/>
+      <c r="F274" s="2" t="n"/>
+    </row>
+    <row r="275">
+      <c r="E275" s="2" t="n"/>
+      <c r="F275" s="2" t="n"/>
+    </row>
+    <row r="276">
+      <c r="E276" s="2" t="n"/>
+      <c r="F276" s="2" t="n"/>
+    </row>
+    <row r="277">
+      <c r="E277" s="2" t="n"/>
+      <c r="F277" s="2" t="n"/>
+    </row>
+    <row r="278">
+      <c r="E278" s="2" t="n"/>
+      <c r="F278" s="2" t="n"/>
+    </row>
+    <row r="279">
+      <c r="E279" s="2" t="n"/>
+      <c r="F279" s="2" t="n"/>
+    </row>
+    <row r="280">
+      <c r="E280" s="2" t="n"/>
+      <c r="F280" s="2" t="n"/>
+    </row>
+    <row r="281">
+      <c r="E281" s="2" t="n"/>
+      <c r="F281" s="2" t="n"/>
+    </row>
+    <row r="282">
+      <c r="E282" s="2" t="n"/>
+      <c r="F282" s="2" t="n"/>
+    </row>
+    <row r="283">
+      <c r="E283" s="2" t="n"/>
+      <c r="F283" s="2" t="n"/>
+    </row>
+    <row r="284">
+      <c r="E284" s="2" t="n"/>
+      <c r="F284" s="2" t="n"/>
+    </row>
+    <row r="285">
+      <c r="E285" s="2" t="n"/>
+      <c r="F285" s="2" t="n"/>
+    </row>
+    <row r="286">
+      <c r="E286" s="2" t="n"/>
+      <c r="F286" s="2" t="n"/>
+    </row>
+    <row r="287">
+      <c r="E287" s="2" t="n"/>
+      <c r="F287" s="2" t="n"/>
+    </row>
+    <row r="288">
+      <c r="E288" s="2" t="n"/>
+      <c r="F288" s="2" t="n"/>
+    </row>
+    <row r="289">
+      <c r="E289" s="2" t="n"/>
+      <c r="F289" s="2" t="n"/>
+    </row>
+    <row r="290">
+      <c r="E290" s="2" t="n"/>
+      <c r="F290" s="2" t="n"/>
+    </row>
+    <row r="291">
+      <c r="E291" s="2" t="n"/>
+      <c r="F291" s="2" t="n"/>
+    </row>
+    <row r="292">
+      <c r="E292" s="2" t="n"/>
+      <c r="F292" s="2" t="n"/>
+    </row>
+    <row r="293">
+      <c r="E293" s="2" t="n"/>
+      <c r="F293" s="2" t="n"/>
+    </row>
+    <row r="294">
+      <c r="E294" s="2" t="n"/>
+      <c r="F294" s="2" t="n"/>
+    </row>
+    <row r="295">
+      <c r="E295" s="2" t="n"/>
+      <c r="F295" s="2" t="n"/>
+    </row>
+    <row r="296">
+      <c r="E296" s="2" t="n"/>
+      <c r="F296" s="2" t="n"/>
+    </row>
+    <row r="297">
+      <c r="E297" s="2" t="n"/>
+      <c r="F297" s="2" t="n"/>
+    </row>
+    <row r="298">
+      <c r="E298" s="2" t="n"/>
+      <c r="F298" s="2" t="n"/>
+    </row>
+    <row r="299">
+      <c r="E299" s="2" t="n"/>
+      <c r="F299" s="2" t="n"/>
+    </row>
+    <row r="300">
+      <c r="E300" s="2" t="n"/>
+      <c r="F300" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>

</xml_diff>

<commit_message>
Intake template: refresh Project dropdown 12 -> 102 current jobs
build_template.py Project list now uses the live Job Board dropdown set
(Name (J####)), regenerated MRA_Project_Intake_Template.xlsx, widened the
column-A validation range. Download now reflects current projects.

https://claude.ai/code/session_01WJTcYohvXPdyiEYiaxvXwj
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -1794,7 +1794,7 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="7">
     <dataValidation sqref="A2:A300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$I$2:$I$13</formula1>
+      <formula1>=Lists!$I$2:$I$103</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$C$2:$C$6</formula1>
@@ -1825,7 +1825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:I31"/>
+  <dimension ref="C1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>2Heads Global Design Ltd (J1548)</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Oakland Schools</t>
+          <t>ABB (J1407)</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Trumpf</t>
+          <t>Aga Kahn Foundation (J1537)</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Age of Union (J1500)</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Washtenaw</t>
+          <t>Amazon (J1513)</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Siemens DI Pedestal</t>
+          <t>Arizona 250 (J1554)</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>SWC HI [CMI]</t>
+          <t>Art Guild (J1563)</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>SMC [Hamilton]</t>
+          <t>ASICS (J1408)</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Thunder Bay MRI Bus</t>
+          <t>AWS (J1217)</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Siemens 53ft Replacement #1</t>
+          <t>Baltimore Aircoil (J1555)</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Siemens 53ft Replacement #2</t>
+          <t>Barton Malow (J1506)</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Stryker</t>
+          <t>Beckman-Coulter-East (J1396)</t>
         </is>
       </c>
     </row>
@@ -2175,6 +2175,11 @@
           <t>Luciana Giglio</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Beckman-Coulter-West (J1396)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="H15" t="inlineStr">
@@ -2182,6 +2187,11 @@
           <t>MRA Design</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Bell Helicopters (J1440)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
@@ -2189,6 +2199,11 @@
           <t>MRA Engineering</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>BioMerieux (J1461)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
@@ -2196,6 +2211,11 @@
           <t>MRA Electrical</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Booz Allen - US Army (J1527)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
@@ -2203,6 +2223,11 @@
           <t>MRA Shop</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Boston Scientific 40ft (J1491)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
@@ -2210,6 +2235,11 @@
           <t>MRA Tech</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Boston Scientific DX (J1507)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="H20" t="inlineStr">
@@ -2217,6 +2247,11 @@
           <t>MRA QA</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Boston Scientific SE (J1496)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="H21" t="inlineStr">
@@ -2224,6 +2259,11 @@
           <t>MRA Ops</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>BPIR Rodeo (J1468)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="H22" t="inlineStr">
@@ -2231,6 +2271,11 @@
           <t>MRA Procurement</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Brain Tumor Foundation (J1481)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="H23" t="inlineStr">
@@ -2238,6 +2283,11 @@
           <t>Art Guild</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Catholic Charities USA (J1538)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="H24" t="inlineStr">
@@ -2245,6 +2295,11 @@
           <t>Art Guild AV</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Cirrus Aircraft (J1549)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="H25" t="inlineStr">
@@ -2252,6 +2307,11 @@
           <t>W2 Graphics</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>CISCO (J1558)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="H26" t="inlineStr">
@@ -2259,6 +2319,11 @@
           <t>Master Wraps</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Climate Action Campaign (J1560)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="H27" t="inlineStr">
@@ -2266,6 +2331,11 @@
           <t>Logistics</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>County of Essex (J1467)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="H28" t="inlineStr">
@@ -2273,6 +2343,11 @@
           <t>Fleet</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Czarnowski (GA) (J1544)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="H29" t="inlineStr">
@@ -2280,6 +2355,11 @@
           <t>Vendor</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>D&amp;G - Canada (J1536)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="H30" t="inlineStr">
@@ -2287,11 +2367,525 @@
           <t>Client</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>D&amp;G - USA Midwest (J1535)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="H31" t="inlineStr">
         <is>
           <t>All</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Duracell (J1383)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Expandable B.V. (J1494)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Ferguson BizBox (J1557)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>FM Global (J1410)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Fortinet III (J1476)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>GRAIL (J1470)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Hershey (J1373)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Hillrom/Baxter (J1445)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Hologic (J1551)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Hyperfine (J1453)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Hyperfine Box Truck #6110 (J1556)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Jewish Federation (J1526)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Knightscope (J1447)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LexCare Hearoes (J1546)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Medtronic (J1553)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Meijer (J1143)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Mkt/Grinder (J1511)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Moon Surgical (J1509)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>MOTT (J1428)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>MRA Internal (J1014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>NHL United by Hockey (J1495)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>NYBC Pod #1 (J1517)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>NYBC Pod #2 (J1531)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>NYBC Pod #3 (J1532)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>NYBC Pod #4 (J1533)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Oakland Schools (J1420)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Oasis Live '25 - The Department (J1539)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Omnicell (J1446)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>On Running (J1559)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>P&amp;G - Tide (J1521)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>PGA of Americas (J1519)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Promaster Retro-Fit (J1775)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>PSE&amp;G / Impact XM (J1508)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>QuidelOrtho (J1384)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Road Show Group (J1774)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>RoadShowGrp / ShowTruckMktng (J1530)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Saskatchewan Health Authority (J1545)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Schaeffler (J1497)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Score (Canada) Limited (J1523)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>SEMI Foundation (J1550)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>SENO Medical (J1454)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>SENO Medical - Box Truck (J1541)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Siemens Big Betty (J1381)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Siemens Canada (J1501)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Siemens Demo Pool (J1209)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Siemens DI (J1524)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Siemens DX #3005 (J1110W)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Siemens DX #92 (J1110E)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Siemens Global Warehousing (J1391)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Siemens Mammo III (J1480)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Siemens Mammo Mandy (J1424)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Sigenergy (J1562)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Simon Wiesenthal Center - MA (Massachusetts) (J1552)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>SMC Corporation (J1542)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Sobeys/Safeway (J1400)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>STI Pod - #1052 (J1561)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Stryker (J1412)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>SWC California (J1486)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>SWC Florida 1 (J1514)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>SWC Florida 2 (J1515)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>SWC Hawaii (J1512)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>SWC Illinois (J1422)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>SWC NY1 (J1487)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>SWC NY2 (J1488)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Tim McGraw (J1421)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Tissot US MotoGP (J1529)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>TravisMathew (J1387)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Warhammer (J1434)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Washtenaw Community College (J1543)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Weill Cornell Imaging (J1540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>WFCU (J1479)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Windsor Champ (J1519)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Winnipeg Regional Health Authority (J1547)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Intake template + import: subtask (Sub) column (rev 3.55)
The intake template now mirrors the master's new Sub column (col O) so
subtasks flow end-to-end:
- build_template.py: adds the Sub column (x/blank dropdown), ships 2
  indented blank subtask slots under each milestone block, with a
  click-prompt explaining the parent→subtask nesting.
- Import-Intake.ps1: MIRROR reader carries the Sub flag and writes it to
  master col O on auto-import (append-only, system columns preserved).
- MRA_Dashboard.html: client-side upload parser + optimistic merge carry
  the Sub flag (importProject payload); download-template cache-buster
  bumped to v=20260618; ? help + CHANGELOG updated.

Pipeline now consistent: template O -> Import-Intake -> master O ->
Export-Data sub -> dashboard editor nesting (rev 3.53).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJTcYohvXPdyiEYiaxvXwj
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -52,7 +52,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -134,6 +139,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -546,6 +555,7 @@
     <col width="26" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -655,6 +665,11 @@
       <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Predecessor</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>Sub</t>
         </is>
       </c>
     </row>
@@ -695,6 +710,7 @@
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9">
@@ -717,6 +733,7 @@
       <c r="L9" s="10" t="n"/>
       <c r="M9" s="9" t="n"/>
       <c r="N9" s="9" t="n"/>
+      <c r="O9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9">
@@ -739,6 +756,7 @@
       <c r="L10" s="10" t="n"/>
       <c r="M10" s="9" t="n"/>
       <c r="N10" s="9" t="n"/>
+      <c r="O10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9">
@@ -761,6 +779,7 @@
       <c r="L11" s="10" t="n"/>
       <c r="M11" s="9" t="n"/>
       <c r="N11" s="9" t="n"/>
+      <c r="O11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9">
@@ -769,7 +788,7 @@
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
+      <c r="D12" s="12" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
       <c r="G12" s="10" t="n"/>
@@ -783,6 +802,11 @@
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="9" t="n"/>
       <c r="N12" s="9" t="n"/>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9">
@@ -791,7 +815,7 @@
       </c>
       <c r="B13" s="10" t="n"/>
       <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
+      <c r="D13" s="12" t="n"/>
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="10" t="n"/>
@@ -805,6 +829,11 @@
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="9" t="n"/>
       <c r="N13" s="9" t="n"/>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7">
@@ -843,6 +872,7 @@
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
+      <c r="O14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9">
@@ -865,6 +895,7 @@
       <c r="L15" s="10" t="n"/>
       <c r="M15" s="9" t="n"/>
       <c r="N15" s="9" t="n"/>
+      <c r="O15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9">
@@ -887,6 +918,7 @@
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="9" t="n"/>
       <c r="N16" s="9" t="n"/>
+      <c r="O16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9">
@@ -909,6 +941,7 @@
       <c r="L17" s="10" t="n"/>
       <c r="M17" s="9" t="n"/>
       <c r="N17" s="9" t="n"/>
+      <c r="O17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9">
@@ -917,7 +950,7 @@
       </c>
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
+      <c r="D18" s="12" t="n"/>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="10" t="n"/>
@@ -931,6 +964,11 @@
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="9" t="n"/>
       <c r="N18" s="9" t="n"/>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9">
@@ -939,7 +977,7 @@
       </c>
       <c r="B19" s="10" t="n"/>
       <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
+      <c r="D19" s="12" t="n"/>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="10" t="n"/>
@@ -953,6 +991,11 @@
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="9" t="n"/>
       <c r="N19" s="9" t="n"/>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7">
@@ -991,6 +1034,7 @@
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9">
@@ -1013,6 +1057,7 @@
       <c r="L21" s="10" t="n"/>
       <c r="M21" s="9" t="n"/>
       <c r="N21" s="9" t="n"/>
+      <c r="O21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9">
@@ -1035,6 +1080,7 @@
       <c r="L22" s="10" t="n"/>
       <c r="M22" s="9" t="n"/>
       <c r="N22" s="9" t="n"/>
+      <c r="O22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9">
@@ -1057,6 +1103,7 @@
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="9" t="n"/>
       <c r="N23" s="9" t="n"/>
+      <c r="O23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9">
@@ -1065,7 +1112,7 @@
       </c>
       <c r="B24" s="10" t="n"/>
       <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
+      <c r="D24" s="12" t="n"/>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="10" t="n"/>
@@ -1079,6 +1126,11 @@
       <c r="L24" s="10" t="n"/>
       <c r="M24" s="9" t="n"/>
       <c r="N24" s="9" t="n"/>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9">
@@ -1087,7 +1139,7 @@
       </c>
       <c r="B25" s="10" t="n"/>
       <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
+      <c r="D25" s="12" t="n"/>
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="10" t="n"/>
@@ -1101,6 +1153,11 @@
       <c r="L25" s="10" t="n"/>
       <c r="M25" s="9" t="n"/>
       <c r="N25" s="9" t="n"/>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7">
@@ -1139,6 +1196,7 @@
       <c r="L26" s="7" t="n"/>
       <c r="M26" s="7" t="n"/>
       <c r="N26" s="7" t="n"/>
+      <c r="O26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9">
@@ -1161,6 +1219,7 @@
       <c r="L27" s="10" t="n"/>
       <c r="M27" s="9" t="n"/>
       <c r="N27" s="9" t="n"/>
+      <c r="O27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9">
@@ -1183,6 +1242,7 @@
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="9" t="n"/>
       <c r="N28" s="9" t="n"/>
+      <c r="O28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9">
@@ -1205,6 +1265,7 @@
       <c r="L29" s="10" t="n"/>
       <c r="M29" s="9" t="n"/>
       <c r="N29" s="9" t="n"/>
+      <c r="O29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9">
@@ -1213,7 +1274,7 @@
       </c>
       <c r="B30" s="10" t="n"/>
       <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
+      <c r="D30" s="12" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="10" t="n"/>
@@ -1227,6 +1288,11 @@
       <c r="L30" s="10" t="n"/>
       <c r="M30" s="9" t="n"/>
       <c r="N30" s="9" t="n"/>
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9">
@@ -1235,7 +1301,7 @@
       </c>
       <c r="B31" s="10" t="n"/>
       <c r="C31" s="10" t="n"/>
-      <c r="D31" s="10" t="n"/>
+      <c r="D31" s="12" t="n"/>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="10" t="n"/>
@@ -1249,6 +1315,11 @@
       <c r="L31" s="10" t="n"/>
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="9" t="n"/>
+      <c r="O31" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7">
@@ -1287,6 +1358,7 @@
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
       <c r="N32" s="7" t="n"/>
+      <c r="O32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9">
@@ -1309,6 +1381,7 @@
       <c r="L33" s="10" t="n"/>
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="9" t="n"/>
+      <c r="O33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9">
@@ -1331,6 +1404,7 @@
       <c r="L34" s="10" t="n"/>
       <c r="M34" s="9" t="n"/>
       <c r="N34" s="9" t="n"/>
+      <c r="O34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9">
@@ -1353,6 +1427,7 @@
       <c r="L35" s="10" t="n"/>
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="9" t="n"/>
+      <c r="O35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="9">
@@ -1361,7 +1436,7 @@
       </c>
       <c r="B36" s="10" t="n"/>
       <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
+      <c r="D36" s="12" t="n"/>
       <c r="E36" s="11" t="n"/>
       <c r="F36" s="11" t="n"/>
       <c r="G36" s="10" t="n"/>
@@ -1375,6 +1450,11 @@
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="9" t="n"/>
+      <c r="O36" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9">
@@ -1383,7 +1463,7 @@
       </c>
       <c r="B37" s="10" t="n"/>
       <c r="C37" s="10" t="n"/>
-      <c r="D37" s="10" t="n"/>
+      <c r="D37" s="12" t="n"/>
       <c r="E37" s="11" t="n"/>
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="10" t="n"/>
@@ -1397,6 +1477,11 @@
       <c r="L37" s="10" t="n"/>
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="9" t="n"/>
+      <c r="O37" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7">
@@ -1435,6 +1520,7 @@
       <c r="L38" s="7" t="n"/>
       <c r="M38" s="7" t="n"/>
       <c r="N38" s="7" t="n"/>
+      <c r="O38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="9">
@@ -1457,6 +1543,7 @@
       <c r="L39" s="10" t="n"/>
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="9" t="n"/>
+      <c r="O39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9">
@@ -1479,6 +1566,7 @@
       <c r="L40" s="10" t="n"/>
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="9" t="n"/>
+      <c r="O40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9">
@@ -1501,6 +1589,7 @@
       <c r="L41" s="10" t="n"/>
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="9" t="n"/>
+      <c r="O41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="9">
@@ -1509,7 +1598,7 @@
       </c>
       <c r="B42" s="10" t="n"/>
       <c r="C42" s="10" t="n"/>
-      <c r="D42" s="10" t="n"/>
+      <c r="D42" s="12" t="n"/>
       <c r="E42" s="11" t="n"/>
       <c r="F42" s="11" t="n"/>
       <c r="G42" s="10" t="n"/>
@@ -1523,6 +1612,11 @@
       <c r="L42" s="10" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="9" t="n"/>
+      <c r="O42" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="9">
@@ -1531,7 +1625,7 @@
       </c>
       <c r="B43" s="10" t="n"/>
       <c r="C43" s="10" t="n"/>
-      <c r="D43" s="10" t="n"/>
+      <c r="D43" s="12" t="n"/>
       <c r="E43" s="11" t="n"/>
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="10" t="n"/>
@@ -1545,6 +1639,11 @@
       <c r="L43" s="10" t="n"/>
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="9" t="n"/>
+      <c r="O43" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7">
@@ -1583,6 +1682,7 @@
       <c r="L44" s="7" t="n"/>
       <c r="M44" s="7" t="n"/>
       <c r="N44" s="7" t="n"/>
+      <c r="O44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9">
@@ -1605,6 +1705,7 @@
       <c r="L45" s="10" t="n"/>
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="9" t="n"/>
+      <c r="O45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9">
@@ -1627,6 +1728,7 @@
       <c r="L46" s="10" t="n"/>
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="9" t="n"/>
+      <c r="O46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9">
@@ -1649,6 +1751,7 @@
       <c r="L47" s="10" t="n"/>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="9" t="n"/>
+      <c r="O47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="9">
@@ -1657,7 +1760,7 @@
       </c>
       <c r="B48" s="10" t="n"/>
       <c r="C48" s="10" t="n"/>
-      <c r="D48" s="10" t="n"/>
+      <c r="D48" s="12" t="n"/>
       <c r="E48" s="11" t="n"/>
       <c r="F48" s="11" t="n"/>
       <c r="G48" s="10" t="n"/>
@@ -1671,6 +1774,11 @@
       <c r="L48" s="10" t="n"/>
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="9" t="n"/>
+      <c r="O48" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9">
@@ -1679,7 +1787,7 @@
       </c>
       <c r="B49" s="10" t="n"/>
       <c r="C49" s="10" t="n"/>
-      <c r="D49" s="10" t="n"/>
+      <c r="D49" s="12" t="n"/>
       <c r="E49" s="11" t="n"/>
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="10" t="n"/>
@@ -1693,6 +1801,11 @@
       <c r="L49" s="10" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="9" t="n"/>
+      <c r="O49" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7">
@@ -1731,6 +1844,7 @@
       <c r="L50" s="7" t="n"/>
       <c r="M50" s="7" t="n"/>
       <c r="N50" s="7" t="n"/>
+      <c r="O50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9">
@@ -1753,6 +1867,7 @@
       <c r="L51" s="10" t="n"/>
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="9" t="n"/>
+      <c r="O51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="9">
@@ -1775,6 +1890,7 @@
       <c r="L52" s="10" t="n"/>
       <c r="M52" s="9" t="n"/>
       <c r="N52" s="9" t="n"/>
+      <c r="O52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9">
@@ -1797,6 +1913,7 @@
       <c r="L53" s="10" t="n"/>
       <c r="M53" s="9" t="n"/>
       <c r="N53" s="9" t="n"/>
+      <c r="O53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="9">
@@ -1805,7 +1922,7 @@
       </c>
       <c r="B54" s="10" t="n"/>
       <c r="C54" s="10" t="n"/>
-      <c r="D54" s="10" t="n"/>
+      <c r="D54" s="12" t="n"/>
       <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
       <c r="G54" s="10" t="n"/>
@@ -1819,6 +1936,11 @@
       <c r="L54" s="10" t="n"/>
       <c r="M54" s="9" t="n"/>
       <c r="N54" s="9" t="n"/>
+      <c r="O54" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9">
@@ -1827,7 +1949,7 @@
       </c>
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="10" t="n"/>
-      <c r="D55" s="10" t="n"/>
+      <c r="D55" s="12" t="n"/>
       <c r="E55" s="11" t="n"/>
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="10" t="n"/>
@@ -1841,6 +1963,11 @@
       <c r="L55" s="10" t="n"/>
       <c r="M55" s="9" t="n"/>
       <c r="N55" s="9" t="n"/>
+      <c r="O55" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7">
@@ -1879,6 +2006,7 @@
       <c r="L56" s="7" t="n"/>
       <c r="M56" s="7" t="n"/>
       <c r="N56" s="7" t="n"/>
+      <c r="O56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9">
@@ -1901,6 +2029,7 @@
       <c r="L57" s="10" t="n"/>
       <c r="M57" s="9" t="n"/>
       <c r="N57" s="9" t="n"/>
+      <c r="O57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="9">
@@ -1923,6 +2052,7 @@
       <c r="L58" s="10" t="n"/>
       <c r="M58" s="9" t="n"/>
       <c r="N58" s="9" t="n"/>
+      <c r="O58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9">
@@ -1945,6 +2075,7 @@
       <c r="L59" s="10" t="n"/>
       <c r="M59" s="9" t="n"/>
       <c r="N59" s="9" t="n"/>
+      <c r="O59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="9">
@@ -1953,7 +2084,7 @@
       </c>
       <c r="B60" s="10" t="n"/>
       <c r="C60" s="10" t="n"/>
-      <c r="D60" s="10" t="n"/>
+      <c r="D60" s="12" t="n"/>
       <c r="E60" s="11" t="n"/>
       <c r="F60" s="11" t="n"/>
       <c r="G60" s="10" t="n"/>
@@ -1967,6 +2098,11 @@
       <c r="L60" s="10" t="n"/>
       <c r="M60" s="9" t="n"/>
       <c r="N60" s="9" t="n"/>
+      <c r="O60" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="9">
@@ -1975,7 +2111,7 @@
       </c>
       <c r="B61" s="10" t="n"/>
       <c r="C61" s="10" t="n"/>
-      <c r="D61" s="10" t="n"/>
+      <c r="D61" s="12" t="n"/>
       <c r="E61" s="11" t="n"/>
       <c r="F61" s="11" t="n"/>
       <c r="G61" s="10" t="n"/>
@@ -1989,6 +2125,11 @@
       <c r="L61" s="10" t="n"/>
       <c r="M61" s="9" t="n"/>
       <c r="N61" s="9" t="n"/>
+      <c r="O61" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7">
@@ -2027,6 +2168,7 @@
       <c r="L62" s="7" t="n"/>
       <c r="M62" s="7" t="n"/>
       <c r="N62" s="7" t="n"/>
+      <c r="O62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9">
@@ -2049,6 +2191,7 @@
       <c r="L63" s="10" t="n"/>
       <c r="M63" s="9" t="n"/>
       <c r="N63" s="9" t="n"/>
+      <c r="O63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="9">
@@ -2071,6 +2214,7 @@
       <c r="L64" s="10" t="n"/>
       <c r="M64" s="9" t="n"/>
       <c r="N64" s="9" t="n"/>
+      <c r="O64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9">
@@ -2093,6 +2237,7 @@
       <c r="L65" s="10" t="n"/>
       <c r="M65" s="9" t="n"/>
       <c r="N65" s="9" t="n"/>
+      <c r="O65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="9">
@@ -2101,7 +2246,7 @@
       </c>
       <c r="B66" s="10" t="n"/>
       <c r="C66" s="10" t="n"/>
-      <c r="D66" s="10" t="n"/>
+      <c r="D66" s="12" t="n"/>
       <c r="E66" s="11" t="n"/>
       <c r="F66" s="11" t="n"/>
       <c r="G66" s="10" t="n"/>
@@ -2115,6 +2260,11 @@
       <c r="L66" s="10" t="n"/>
       <c r="M66" s="9" t="n"/>
       <c r="N66" s="9" t="n"/>
+      <c r="O66" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="9">
@@ -2123,7 +2273,7 @@
       </c>
       <c r="B67" s="10" t="n"/>
       <c r="C67" s="10" t="n"/>
-      <c r="D67" s="10" t="n"/>
+      <c r="D67" s="12" t="n"/>
       <c r="E67" s="11" t="n"/>
       <c r="F67" s="11" t="n"/>
       <c r="G67" s="10" t="n"/>
@@ -2137,6 +2287,11 @@
       <c r="L67" s="10" t="n"/>
       <c r="M67" s="9" t="n"/>
       <c r="N67" s="9" t="n"/>
+      <c r="O67" s="13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="9">
@@ -2159,6 +2314,7 @@
       <c r="L68" s="10" t="n"/>
       <c r="M68" s="9" t="n"/>
       <c r="N68" s="9" t="n"/>
+      <c r="O68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9">
@@ -2181,6 +2337,7 @@
       <c r="L69" s="10" t="n"/>
       <c r="M69" s="9" t="n"/>
       <c r="N69" s="9" t="n"/>
+      <c r="O69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="9">
@@ -2203,6 +2360,7 @@
       <c r="L70" s="10" t="n"/>
       <c r="M70" s="9" t="n"/>
       <c r="N70" s="9" t="n"/>
+      <c r="O70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9">
@@ -2225,6 +2383,7 @@
       <c r="L71" s="10" t="n"/>
       <c r="M71" s="9" t="n"/>
       <c r="N71" s="9" t="n"/>
+      <c r="O71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9">
@@ -2247,6 +2406,7 @@
       <c r="L72" s="10" t="n"/>
       <c r="M72" s="9" t="n"/>
       <c r="N72" s="9" t="n"/>
+      <c r="O72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9">
@@ -2269,6 +2429,7 @@
       <c r="L73" s="10" t="n"/>
       <c r="M73" s="9" t="n"/>
       <c r="N73" s="9" t="n"/>
+      <c r="O73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9">
@@ -2291,6 +2452,7 @@
       <c r="L74" s="10" t="n"/>
       <c r="M74" s="9" t="n"/>
       <c r="N74" s="9" t="n"/>
+      <c r="O74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9">
@@ -2313,6 +2475,7 @@
       <c r="L75" s="10" t="n"/>
       <c r="M75" s="9" t="n"/>
       <c r="N75" s="9" t="n"/>
+      <c r="O75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="9">
@@ -2335,6 +2498,7 @@
       <c r="L76" s="10" t="n"/>
       <c r="M76" s="9" t="n"/>
       <c r="N76" s="9" t="n"/>
+      <c r="O76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9">
@@ -2357,6 +2521,7 @@
       <c r="L77" s="10" t="n"/>
       <c r="M77" s="9" t="n"/>
       <c r="N77" s="9" t="n"/>
+      <c r="O77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="9">
@@ -2379,6 +2544,7 @@
       <c r="L78" s="10" t="n"/>
       <c r="M78" s="9" t="n"/>
       <c r="N78" s="9" t="n"/>
+      <c r="O78" s="10" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9">
@@ -2401,6 +2567,7 @@
       <c r="L79" s="10" t="n"/>
       <c r="M79" s="9" t="n"/>
       <c r="N79" s="9" t="n"/>
+      <c r="O79" s="10" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="9">
@@ -2423,6 +2590,7 @@
       <c r="L80" s="10" t="n"/>
       <c r="M80" s="9" t="n"/>
       <c r="N80" s="9" t="n"/>
+      <c r="O80" s="10" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9">
@@ -2445,6 +2613,7 @@
       <c r="L81" s="10" t="n"/>
       <c r="M81" s="9" t="n"/>
       <c r="N81" s="9" t="n"/>
+      <c r="O81" s="10" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="9">
@@ -2467,6 +2636,7 @@
       <c r="L82" s="10" t="n"/>
       <c r="M82" s="9" t="n"/>
       <c r="N82" s="9" t="n"/>
+      <c r="O82" s="10" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9">
@@ -2489,6 +2659,7 @@
       <c r="L83" s="10" t="n"/>
       <c r="M83" s="9" t="n"/>
       <c r="N83" s="9" t="n"/>
+      <c r="O83" s="10" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="9">
@@ -2511,6 +2682,7 @@
       <c r="L84" s="10" t="n"/>
       <c r="M84" s="9" t="n"/>
       <c r="N84" s="9" t="n"/>
+      <c r="O84" s="10" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9">
@@ -2533,6 +2705,7 @@
       <c r="L85" s="10" t="n"/>
       <c r="M85" s="9" t="n"/>
       <c r="N85" s="9" t="n"/>
+      <c r="O85" s="10" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="9">
@@ -2555,6 +2728,7 @@
       <c r="L86" s="10" t="n"/>
       <c r="M86" s="9" t="n"/>
       <c r="N86" s="9" t="n"/>
+      <c r="O86" s="10" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9">
@@ -2577,6 +2751,7 @@
       <c r="L87" s="10" t="n"/>
       <c r="M87" s="9" t="n"/>
       <c r="N87" s="9" t="n"/>
+      <c r="O87" s="10" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="9">
@@ -2599,6 +2774,7 @@
       <c r="L88" s="10" t="n"/>
       <c r="M88" s="9" t="n"/>
       <c r="N88" s="9" t="n"/>
+      <c r="O88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9">
@@ -2621,6 +2797,7 @@
       <c r="L89" s="10" t="n"/>
       <c r="M89" s="9" t="n"/>
       <c r="N89" s="9" t="n"/>
+      <c r="O89" s="10" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="9">
@@ -2643,6 +2820,7 @@
       <c r="L90" s="10" t="n"/>
       <c r="M90" s="9" t="n"/>
       <c r="N90" s="9" t="n"/>
+      <c r="O90" s="10" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="9">
@@ -2665,6 +2843,7 @@
       <c r="L91" s="10" t="n"/>
       <c r="M91" s="9" t="n"/>
       <c r="N91" s="9" t="n"/>
+      <c r="O91" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="9">
@@ -2687,6 +2866,7 @@
       <c r="L92" s="10" t="n"/>
       <c r="M92" s="9" t="n"/>
       <c r="N92" s="9" t="n"/>
+      <c r="O92" s="10" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9">
@@ -2709,6 +2889,7 @@
       <c r="L93" s="10" t="n"/>
       <c r="M93" s="9" t="n"/>
       <c r="N93" s="9" t="n"/>
+      <c r="O93" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="9">
@@ -2731,6 +2912,7 @@
       <c r="L94" s="10" t="n"/>
       <c r="M94" s="9" t="n"/>
       <c r="N94" s="9" t="n"/>
+      <c r="O94" s="10" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="9">
@@ -2753,6 +2935,7 @@
       <c r="L95" s="10" t="n"/>
       <c r="M95" s="9" t="n"/>
       <c r="N95" s="9" t="n"/>
+      <c r="O95" s="10" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="9">
@@ -2775,6 +2958,7 @@
       <c r="L96" s="10" t="n"/>
       <c r="M96" s="9" t="n"/>
       <c r="N96" s="9" t="n"/>
+      <c r="O96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="9">
@@ -2797,6 +2981,7 @@
       <c r="L97" s="10" t="n"/>
       <c r="M97" s="9" t="n"/>
       <c r="N97" s="9" t="n"/>
+      <c r="O97" s="10" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="9">
@@ -2819,6 +3004,7 @@
       <c r="L98" s="10" t="n"/>
       <c r="M98" s="9" t="n"/>
       <c r="N98" s="9" t="n"/>
+      <c r="O98" s="10" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="9">
@@ -2841,6 +3027,7 @@
       <c r="L99" s="10" t="n"/>
       <c r="M99" s="9" t="n"/>
       <c r="N99" s="9" t="n"/>
+      <c r="O99" s="10" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="9">
@@ -2863,6 +3050,7 @@
       <c r="L100" s="10" t="n"/>
       <c r="M100" s="9" t="n"/>
       <c r="N100" s="9" t="n"/>
+      <c r="O100" s="10" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="9">
@@ -2885,6 +3073,7 @@
       <c r="L101" s="10" t="n"/>
       <c r="M101" s="9" t="n"/>
       <c r="N101" s="9" t="n"/>
+      <c r="O101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="9">
@@ -2907,6 +3096,7 @@
       <c r="L102" s="10" t="n"/>
       <c r="M102" s="9" t="n"/>
       <c r="N102" s="9" t="n"/>
+      <c r="O102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="9">
@@ -2929,6 +3119,7 @@
       <c r="L103" s="10" t="n"/>
       <c r="M103" s="9" t="n"/>
       <c r="N103" s="9" t="n"/>
+      <c r="O103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="9">
@@ -2951,6 +3142,7 @@
       <c r="L104" s="10" t="n"/>
       <c r="M104" s="9" t="n"/>
       <c r="N104" s="9" t="n"/>
+      <c r="O104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="9">
@@ -2973,6 +3165,7 @@
       <c r="L105" s="10" t="n"/>
       <c r="M105" s="9" t="n"/>
       <c r="N105" s="9" t="n"/>
+      <c r="O105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="9">
@@ -2995,6 +3188,7 @@
       <c r="L106" s="10" t="n"/>
       <c r="M106" s="9" t="n"/>
       <c r="N106" s="9" t="n"/>
+      <c r="O106" s="10" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="9">
@@ -3017,6 +3211,7 @@
       <c r="L107" s="10" t="n"/>
       <c r="M107" s="9" t="n"/>
       <c r="N107" s="9" t="n"/>
+      <c r="O107" s="10" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="9">
@@ -3039,6 +3234,7 @@
       <c r="L108" s="10" t="n"/>
       <c r="M108" s="9" t="n"/>
       <c r="N108" s="9" t="n"/>
+      <c r="O108" s="10" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="9">
@@ -3061,6 +3257,7 @@
       <c r="L109" s="10" t="n"/>
       <c r="M109" s="9" t="n"/>
       <c r="N109" s="9" t="n"/>
+      <c r="O109" s="10" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="9">
@@ -3083,6 +3280,7 @@
       <c r="L110" s="10" t="n"/>
       <c r="M110" s="9" t="n"/>
       <c r="N110" s="9" t="n"/>
+      <c r="O110" s="10" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="9">
@@ -3105,6 +3303,7 @@
       <c r="L111" s="10" t="n"/>
       <c r="M111" s="9" t="n"/>
       <c r="N111" s="9" t="n"/>
+      <c r="O111" s="10" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="9">
@@ -3127,6 +3326,7 @@
       <c r="L112" s="10" t="n"/>
       <c r="M112" s="9" t="n"/>
       <c r="N112" s="9" t="n"/>
+      <c r="O112" s="10" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="9">
@@ -3149,6 +3349,7 @@
       <c r="L113" s="10" t="n"/>
       <c r="M113" s="9" t="n"/>
       <c r="N113" s="9" t="n"/>
+      <c r="O113" s="10" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="9">
@@ -3171,6 +3372,7 @@
       <c r="L114" s="10" t="n"/>
       <c r="M114" s="9" t="n"/>
       <c r="N114" s="9" t="n"/>
+      <c r="O114" s="10" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="9">
@@ -3193,6 +3395,7 @@
       <c r="L115" s="10" t="n"/>
       <c r="M115" s="9" t="n"/>
       <c r="N115" s="9" t="n"/>
+      <c r="O115" s="10" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="9">
@@ -3215,6 +3418,7 @@
       <c r="L116" s="10" t="n"/>
       <c r="M116" s="9" t="n"/>
       <c r="N116" s="9" t="n"/>
+      <c r="O116" s="10" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="9">
@@ -3237,6 +3441,7 @@
       <c r="L117" s="10" t="n"/>
       <c r="M117" s="9" t="n"/>
       <c r="N117" s="9" t="n"/>
+      <c r="O117" s="10" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="9">
@@ -3259,6 +3464,7 @@
       <c r="L118" s="10" t="n"/>
       <c r="M118" s="9" t="n"/>
       <c r="N118" s="9" t="n"/>
+      <c r="O118" s="10" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="9">
@@ -3281,6 +3487,7 @@
       <c r="L119" s="10" t="n"/>
       <c r="M119" s="9" t="n"/>
       <c r="N119" s="9" t="n"/>
+      <c r="O119" s="10" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="9">
@@ -3303,6 +3510,7 @@
       <c r="L120" s="10" t="n"/>
       <c r="M120" s="9" t="n"/>
       <c r="N120" s="9" t="n"/>
+      <c r="O120" s="10" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="9">
@@ -3325,6 +3533,7 @@
       <c r="L121" s="10" t="n"/>
       <c r="M121" s="9" t="n"/>
       <c r="N121" s="9" t="n"/>
+      <c r="O121" s="10" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="9">
@@ -3347,6 +3556,7 @@
       <c r="L122" s="10" t="n"/>
       <c r="M122" s="9" t="n"/>
       <c r="N122" s="9" t="n"/>
+      <c r="O122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="9">
@@ -3369,6 +3579,7 @@
       <c r="L123" s="10" t="n"/>
       <c r="M123" s="9" t="n"/>
       <c r="N123" s="9" t="n"/>
+      <c r="O123" s="10" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="9">
@@ -3391,6 +3602,7 @@
       <c r="L124" s="10" t="n"/>
       <c r="M124" s="9" t="n"/>
       <c r="N124" s="9" t="n"/>
+      <c r="O124" s="10" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="9">
@@ -3413,6 +3625,7 @@
       <c r="L125" s="10" t="n"/>
       <c r="M125" s="9" t="n"/>
       <c r="N125" s="9" t="n"/>
+      <c r="O125" s="10" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="9">
@@ -3435,6 +3648,7 @@
       <c r="L126" s="10" t="n"/>
       <c r="M126" s="9" t="n"/>
       <c r="N126" s="9" t="n"/>
+      <c r="O126" s="10" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="9">
@@ -3457,19 +3671,21 @@
       <c r="L127" s="10" t="n"/>
       <c r="M127" s="9" t="n"/>
       <c r="N127" s="9" t="n"/>
+      <c r="O127" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="C2:N2"/>
-    <mergeCell ref="C1:N1"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="C1:O1"/>
+    <mergeCell ref="C2:O2"/>
   </mergeCells>
-  <dataValidations count="9">
+  <dataValidations count="11">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Project / Client" prompt="Type the project name (new jobs welcome). It auto-fills down column A."/>
     <dataValidation sqref="G4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="MRA Job #" prompt="Job number if you have one, or type &quot;NEW&quot;."/>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Project Manager" prompt="The PM for this project — auto-fills down column J."/>
+    <dataValidation sqref="D12 D13 D18 D19 D24 D25 D30 D31 D36 D37 D42 D43 D48 D49 D54 D55 D60 D61 D66 D67" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Subtask" prompt="Subtask of the task above. Type the subtask here and keep the &quot;x&quot; in the Sub column — the dashboard nests it (collapsible) under its parent. Clear the &quot;x&quot; to make it a normal task."/>
     <dataValidation sqref="B8:B127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$B$2:$B$10</formula1>
     </dataValidation>
@@ -3484,6 +3700,9 @@
     </dataValidation>
     <dataValidation sqref="K8:K127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$E$2:$E$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="O8:O127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Lists!$H$2:$H$2</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$F$2:$F$14</formula1>
@@ -3502,7 +3721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G19"/>
+  <dimension ref="B1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3536,6 +3755,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -3566,6 +3790,11 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>MRA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sub-resources: two-level Resource Schedule (group › person) + workbook column (rev 3.66)
Dashboard: Crew/Resource Schedule picker is now two-level via taskLanes() —
each group (MRA Design, MRA Shop, Electricians, Wrap Team, Maintenance) rolls
up everyone ("MRA Design — all") with members indented ("› Steve K") as
<optgroup>s; standalones go under "People / Other". CREW_ALIAS is now
group-name normalization only (persons become members, not folded away).
Member = the new Sub-Resource column when present, else the non-group half of
an "A / B" assignment, so it works on existing data today.

Workbook side: Export-Data.ps1 reads Sub-Resource (col P) -> emits subRes;
build_template.py + the intake template add a Sub-Resource column (P) with an
input-message prompt. Download cache-buster -> v=20260618c. Help + CHANGELOG.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJTcYohvXPdyiEYiaxvXwj
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O129"/>
+  <dimension ref="A1:P129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,7 @@
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -621,6 +622,7 @@
       <c r="M6" s="6" t="n"/>
       <c r="N6" s="6" t="n"/>
       <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -642,6 +644,7 @@
       <c r="M7" s="6" t="n"/>
       <c r="N7" s="6" t="n"/>
       <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
     </row>
     <row r="8" ht="8" customHeight="1"/>
     <row r="9" ht="24" customHeight="1">
@@ -718,6 +721,11 @@
       <c r="O9" s="9" t="inlineStr">
         <is>
           <t>Sub</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>Sub-Resource</t>
         </is>
       </c>
     </row>
@@ -759,6 +767,7 @@
       <c r="M10" s="10" t="n"/>
       <c r="N10" s="10" t="n"/>
       <c r="O10" s="10" t="n"/>
+      <c r="P10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12">
@@ -782,6 +791,7 @@
       <c r="M11" s="12" t="n"/>
       <c r="N11" s="12" t="n"/>
       <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12">
@@ -805,6 +815,7 @@
       <c r="M12" s="12" t="n"/>
       <c r="N12" s="12" t="n"/>
       <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12">
@@ -828,6 +839,7 @@
       <c r="M13" s="12" t="n"/>
       <c r="N13" s="12" t="n"/>
       <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12">
@@ -855,6 +867,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12">
@@ -882,6 +895,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10">
@@ -921,6 +935,7 @@
       <c r="M16" s="10" t="n"/>
       <c r="N16" s="10" t="n"/>
       <c r="O16" s="10" t="n"/>
+      <c r="P16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12">
@@ -944,6 +959,7 @@
       <c r="M17" s="12" t="n"/>
       <c r="N17" s="12" t="n"/>
       <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12">
@@ -967,6 +983,7 @@
       <c r="M18" s="12" t="n"/>
       <c r="N18" s="12" t="n"/>
       <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12">
@@ -990,6 +1007,7 @@
       <c r="M19" s="12" t="n"/>
       <c r="N19" s="12" t="n"/>
       <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12">
@@ -1017,6 +1035,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12">
@@ -1044,6 +1063,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10">
@@ -1083,6 +1103,7 @@
       <c r="M22" s="10" t="n"/>
       <c r="N22" s="10" t="n"/>
       <c r="O22" s="10" t="n"/>
+      <c r="P22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12">
@@ -1106,6 +1127,7 @@
       <c r="M23" s="12" t="n"/>
       <c r="N23" s="12" t="n"/>
       <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="12">
@@ -1129,6 +1151,7 @@
       <c r="M24" s="12" t="n"/>
       <c r="N24" s="12" t="n"/>
       <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12">
@@ -1152,6 +1175,7 @@
       <c r="M25" s="12" t="n"/>
       <c r="N25" s="12" t="n"/>
       <c r="O25" s="6" t="n"/>
+      <c r="P25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12">
@@ -1179,6 +1203,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="12">
@@ -1206,6 +1231,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10">
@@ -1245,6 +1271,7 @@
       <c r="M28" s="10" t="n"/>
       <c r="N28" s="10" t="n"/>
       <c r="O28" s="10" t="n"/>
+      <c r="P28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12">
@@ -1268,6 +1295,7 @@
       <c r="M29" s="12" t="n"/>
       <c r="N29" s="12" t="n"/>
       <c r="O29" s="6" t="n"/>
+      <c r="P29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12">
@@ -1291,6 +1319,7 @@
       <c r="M30" s="12" t="n"/>
       <c r="N30" s="12" t="n"/>
       <c r="O30" s="6" t="n"/>
+      <c r="P30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12">
@@ -1314,6 +1343,7 @@
       <c r="M31" s="12" t="n"/>
       <c r="N31" s="12" t="n"/>
       <c r="O31" s="6" t="n"/>
+      <c r="P31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12">
@@ -1341,6 +1371,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12">
@@ -1368,6 +1399,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10">
@@ -1407,6 +1439,7 @@
       <c r="M34" s="10" t="n"/>
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
+      <c r="P34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12">
@@ -1430,6 +1463,7 @@
       <c r="M35" s="12" t="n"/>
       <c r="N35" s="12" t="n"/>
       <c r="O35" s="6" t="n"/>
+      <c r="P35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12">
@@ -1453,6 +1487,7 @@
       <c r="M36" s="12" t="n"/>
       <c r="N36" s="12" t="n"/>
       <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12">
@@ -1476,6 +1511,7 @@
       <c r="M37" s="12" t="n"/>
       <c r="N37" s="12" t="n"/>
       <c r="O37" s="6" t="n"/>
+      <c r="P37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="12">
@@ -1503,6 +1539,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12">
@@ -1530,6 +1567,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10">
@@ -1569,6 +1607,7 @@
       <c r="M40" s="10" t="n"/>
       <c r="N40" s="10" t="n"/>
       <c r="O40" s="10" t="n"/>
+      <c r="P40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12">
@@ -1592,6 +1631,7 @@
       <c r="M41" s="12" t="n"/>
       <c r="N41" s="12" t="n"/>
       <c r="O41" s="6" t="n"/>
+      <c r="P41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12">
@@ -1615,6 +1655,7 @@
       <c r="M42" s="12" t="n"/>
       <c r="N42" s="12" t="n"/>
       <c r="O42" s="6" t="n"/>
+      <c r="P42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="12">
@@ -1638,6 +1679,7 @@
       <c r="M43" s="12" t="n"/>
       <c r="N43" s="12" t="n"/>
       <c r="O43" s="6" t="n"/>
+      <c r="P43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12">
@@ -1665,6 +1707,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="12">
@@ -1692,6 +1735,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10">
@@ -1731,6 +1775,7 @@
       <c r="M46" s="10" t="n"/>
       <c r="N46" s="10" t="n"/>
       <c r="O46" s="10" t="n"/>
+      <c r="P46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="12">
@@ -1754,6 +1799,7 @@
       <c r="M47" s="12" t="n"/>
       <c r="N47" s="12" t="n"/>
       <c r="O47" s="6" t="n"/>
+      <c r="P47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="12">
@@ -1777,6 +1823,7 @@
       <c r="M48" s="12" t="n"/>
       <c r="N48" s="12" t="n"/>
       <c r="O48" s="6" t="n"/>
+      <c r="P48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="12">
@@ -1800,6 +1847,7 @@
       <c r="M49" s="12" t="n"/>
       <c r="N49" s="12" t="n"/>
       <c r="O49" s="6" t="n"/>
+      <c r="P49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="12">
@@ -1827,6 +1875,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="12">
@@ -1854,6 +1903,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10">
@@ -1893,6 +1943,7 @@
       <c r="M52" s="10" t="n"/>
       <c r="N52" s="10" t="n"/>
       <c r="O52" s="10" t="n"/>
+      <c r="P52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="12">
@@ -1916,6 +1967,7 @@
       <c r="M53" s="12" t="n"/>
       <c r="N53" s="12" t="n"/>
       <c r="O53" s="6" t="n"/>
+      <c r="P53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="12">
@@ -1939,6 +1991,7 @@
       <c r="M54" s="12" t="n"/>
       <c r="N54" s="12" t="n"/>
       <c r="O54" s="6" t="n"/>
+      <c r="P54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="12">
@@ -1962,6 +2015,7 @@
       <c r="M55" s="12" t="n"/>
       <c r="N55" s="12" t="n"/>
       <c r="O55" s="6" t="n"/>
+      <c r="P55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="12">
@@ -1989,6 +2043,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="12">
@@ -2016,6 +2071,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10">
@@ -2055,6 +2111,7 @@
       <c r="M58" s="10" t="n"/>
       <c r="N58" s="10" t="n"/>
       <c r="O58" s="10" t="n"/>
+      <c r="P58" s="10" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="12">
@@ -2078,6 +2135,7 @@
       <c r="M59" s="12" t="n"/>
       <c r="N59" s="12" t="n"/>
       <c r="O59" s="6" t="n"/>
+      <c r="P59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12">
@@ -2101,6 +2159,7 @@
       <c r="M60" s="12" t="n"/>
       <c r="N60" s="12" t="n"/>
       <c r="O60" s="6" t="n"/>
+      <c r="P60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="12">
@@ -2124,6 +2183,7 @@
       <c r="M61" s="12" t="n"/>
       <c r="N61" s="12" t="n"/>
       <c r="O61" s="6" t="n"/>
+      <c r="P61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12">
@@ -2151,6 +2211,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="12">
@@ -2178,6 +2239,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10">
@@ -2217,6 +2279,7 @@
       <c r="M64" s="10" t="n"/>
       <c r="N64" s="10" t="n"/>
       <c r="O64" s="10" t="n"/>
+      <c r="P64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="12">
@@ -2240,6 +2303,7 @@
       <c r="M65" s="12" t="n"/>
       <c r="N65" s="12" t="n"/>
       <c r="O65" s="6" t="n"/>
+      <c r="P65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="12">
@@ -2263,6 +2327,7 @@
       <c r="M66" s="12" t="n"/>
       <c r="N66" s="12" t="n"/>
       <c r="O66" s="6" t="n"/>
+      <c r="P66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="12">
@@ -2286,6 +2351,7 @@
       <c r="M67" s="12" t="n"/>
       <c r="N67" s="12" t="n"/>
       <c r="O67" s="6" t="n"/>
+      <c r="P67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="12">
@@ -2313,6 +2379,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="12">
@@ -2340,6 +2407,7 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="12">
@@ -2363,6 +2431,7 @@
       <c r="M70" s="12" t="n"/>
       <c r="N70" s="12" t="n"/>
       <c r="O70" s="6" t="n"/>
+      <c r="P70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="12">
@@ -2386,6 +2455,7 @@
       <c r="M71" s="12" t="n"/>
       <c r="N71" s="12" t="n"/>
       <c r="O71" s="6" t="n"/>
+      <c r="P71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="12">
@@ -2409,6 +2479,7 @@
       <c r="M72" s="12" t="n"/>
       <c r="N72" s="12" t="n"/>
       <c r="O72" s="6" t="n"/>
+      <c r="P72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="12">
@@ -2432,6 +2503,7 @@
       <c r="M73" s="12" t="n"/>
       <c r="N73" s="12" t="n"/>
       <c r="O73" s="6" t="n"/>
+      <c r="P73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="12">
@@ -2455,6 +2527,7 @@
       <c r="M74" s="12" t="n"/>
       <c r="N74" s="12" t="n"/>
       <c r="O74" s="6" t="n"/>
+      <c r="P74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="12">
@@ -2478,6 +2551,7 @@
       <c r="M75" s="12" t="n"/>
       <c r="N75" s="12" t="n"/>
       <c r="O75" s="6" t="n"/>
+      <c r="P75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="12">
@@ -2501,6 +2575,7 @@
       <c r="M76" s="12" t="n"/>
       <c r="N76" s="12" t="n"/>
       <c r="O76" s="6" t="n"/>
+      <c r="P76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="12">
@@ -2524,6 +2599,7 @@
       <c r="M77" s="12" t="n"/>
       <c r="N77" s="12" t="n"/>
       <c r="O77" s="6" t="n"/>
+      <c r="P77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="12">
@@ -2547,6 +2623,7 @@
       <c r="M78" s="12" t="n"/>
       <c r="N78" s="12" t="n"/>
       <c r="O78" s="6" t="n"/>
+      <c r="P78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="12">
@@ -2570,6 +2647,7 @@
       <c r="M79" s="12" t="n"/>
       <c r="N79" s="12" t="n"/>
       <c r="O79" s="6" t="n"/>
+      <c r="P79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="12">
@@ -2593,6 +2671,7 @@
       <c r="M80" s="12" t="n"/>
       <c r="N80" s="12" t="n"/>
       <c r="O80" s="6" t="n"/>
+      <c r="P80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="12">
@@ -2616,6 +2695,7 @@
       <c r="M81" s="12" t="n"/>
       <c r="N81" s="12" t="n"/>
       <c r="O81" s="6" t="n"/>
+      <c r="P81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="12">
@@ -2639,6 +2719,7 @@
       <c r="M82" s="12" t="n"/>
       <c r="N82" s="12" t="n"/>
       <c r="O82" s="6" t="n"/>
+      <c r="P82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="12">
@@ -2662,6 +2743,7 @@
       <c r="M83" s="12" t="n"/>
       <c r="N83" s="12" t="n"/>
       <c r="O83" s="6" t="n"/>
+      <c r="P83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="12">
@@ -2685,6 +2767,7 @@
       <c r="M84" s="12" t="n"/>
       <c r="N84" s="12" t="n"/>
       <c r="O84" s="6" t="n"/>
+      <c r="P84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="12">
@@ -2708,6 +2791,7 @@
       <c r="M85" s="12" t="n"/>
       <c r="N85" s="12" t="n"/>
       <c r="O85" s="6" t="n"/>
+      <c r="P85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="12">
@@ -2731,6 +2815,7 @@
       <c r="M86" s="12" t="n"/>
       <c r="N86" s="12" t="n"/>
       <c r="O86" s="6" t="n"/>
+      <c r="P86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="12">
@@ -2754,6 +2839,7 @@
       <c r="M87" s="12" t="n"/>
       <c r="N87" s="12" t="n"/>
       <c r="O87" s="6" t="n"/>
+      <c r="P87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="12">
@@ -2777,6 +2863,7 @@
       <c r="M88" s="12" t="n"/>
       <c r="N88" s="12" t="n"/>
       <c r="O88" s="6" t="n"/>
+      <c r="P88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="12">
@@ -2800,6 +2887,7 @@
       <c r="M89" s="12" t="n"/>
       <c r="N89" s="12" t="n"/>
       <c r="O89" s="6" t="n"/>
+      <c r="P89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="12">
@@ -2823,6 +2911,7 @@
       <c r="M90" s="12" t="n"/>
       <c r="N90" s="12" t="n"/>
       <c r="O90" s="6" t="n"/>
+      <c r="P90" s="6" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="12">
@@ -2846,6 +2935,7 @@
       <c r="M91" s="12" t="n"/>
       <c r="N91" s="12" t="n"/>
       <c r="O91" s="6" t="n"/>
+      <c r="P91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="12">
@@ -2869,6 +2959,7 @@
       <c r="M92" s="12" t="n"/>
       <c r="N92" s="12" t="n"/>
       <c r="O92" s="6" t="n"/>
+      <c r="P92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="12">
@@ -2892,6 +2983,7 @@
       <c r="M93" s="12" t="n"/>
       <c r="N93" s="12" t="n"/>
       <c r="O93" s="6" t="n"/>
+      <c r="P93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="12">
@@ -2915,6 +3007,7 @@
       <c r="M94" s="12" t="n"/>
       <c r="N94" s="12" t="n"/>
       <c r="O94" s="6" t="n"/>
+      <c r="P94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="12">
@@ -2938,6 +3031,7 @@
       <c r="M95" s="12" t="n"/>
       <c r="N95" s="12" t="n"/>
       <c r="O95" s="6" t="n"/>
+      <c r="P95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="12">
@@ -2961,6 +3055,7 @@
       <c r="M96" s="12" t="n"/>
       <c r="N96" s="12" t="n"/>
       <c r="O96" s="6" t="n"/>
+      <c r="P96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="12">
@@ -2984,6 +3079,7 @@
       <c r="M97" s="12" t="n"/>
       <c r="N97" s="12" t="n"/>
       <c r="O97" s="6" t="n"/>
+      <c r="P97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="12">
@@ -3007,6 +3103,7 @@
       <c r="M98" s="12" t="n"/>
       <c r="N98" s="12" t="n"/>
       <c r="O98" s="6" t="n"/>
+      <c r="P98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="12">
@@ -3030,6 +3127,7 @@
       <c r="M99" s="12" t="n"/>
       <c r="N99" s="12" t="n"/>
       <c r="O99" s="6" t="n"/>
+      <c r="P99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="12">
@@ -3053,6 +3151,7 @@
       <c r="M100" s="12" t="n"/>
       <c r="N100" s="12" t="n"/>
       <c r="O100" s="6" t="n"/>
+      <c r="P100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="12">
@@ -3076,6 +3175,7 @@
       <c r="M101" s="12" t="n"/>
       <c r="N101" s="12" t="n"/>
       <c r="O101" s="6" t="n"/>
+      <c r="P101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="12">
@@ -3099,6 +3199,7 @@
       <c r="M102" s="12" t="n"/>
       <c r="N102" s="12" t="n"/>
       <c r="O102" s="6" t="n"/>
+      <c r="P102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="12">
@@ -3122,6 +3223,7 @@
       <c r="M103" s="12" t="n"/>
       <c r="N103" s="12" t="n"/>
       <c r="O103" s="6" t="n"/>
+      <c r="P103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="12">
@@ -3145,6 +3247,7 @@
       <c r="M104" s="12" t="n"/>
       <c r="N104" s="12" t="n"/>
       <c r="O104" s="6" t="n"/>
+      <c r="P104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="12">
@@ -3168,6 +3271,7 @@
       <c r="M105" s="12" t="n"/>
       <c r="N105" s="12" t="n"/>
       <c r="O105" s="6" t="n"/>
+      <c r="P105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="12">
@@ -3191,6 +3295,7 @@
       <c r="M106" s="12" t="n"/>
       <c r="N106" s="12" t="n"/>
       <c r="O106" s="6" t="n"/>
+      <c r="P106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="12">
@@ -3214,6 +3319,7 @@
       <c r="M107" s="12" t="n"/>
       <c r="N107" s="12" t="n"/>
       <c r="O107" s="6" t="n"/>
+      <c r="P107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="12">
@@ -3237,6 +3343,7 @@
       <c r="M108" s="12" t="n"/>
       <c r="N108" s="12" t="n"/>
       <c r="O108" s="6" t="n"/>
+      <c r="P108" s="6" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="12">
@@ -3260,6 +3367,7 @@
       <c r="M109" s="12" t="n"/>
       <c r="N109" s="12" t="n"/>
       <c r="O109" s="6" t="n"/>
+      <c r="P109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="12">
@@ -3283,6 +3391,7 @@
       <c r="M110" s="12" t="n"/>
       <c r="N110" s="12" t="n"/>
       <c r="O110" s="6" t="n"/>
+      <c r="P110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="12">
@@ -3306,6 +3415,7 @@
       <c r="M111" s="12" t="n"/>
       <c r="N111" s="12" t="n"/>
       <c r="O111" s="6" t="n"/>
+      <c r="P111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="12">
@@ -3329,6 +3439,7 @@
       <c r="M112" s="12" t="n"/>
       <c r="N112" s="12" t="n"/>
       <c r="O112" s="6" t="n"/>
+      <c r="P112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="12">
@@ -3352,6 +3463,7 @@
       <c r="M113" s="12" t="n"/>
       <c r="N113" s="12" t="n"/>
       <c r="O113" s="6" t="n"/>
+      <c r="P113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="12">
@@ -3375,6 +3487,7 @@
       <c r="M114" s="12" t="n"/>
       <c r="N114" s="12" t="n"/>
       <c r="O114" s="6" t="n"/>
+      <c r="P114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="12">
@@ -3398,6 +3511,7 @@
       <c r="M115" s="12" t="n"/>
       <c r="N115" s="12" t="n"/>
       <c r="O115" s="6" t="n"/>
+      <c r="P115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="12">
@@ -3421,6 +3535,7 @@
       <c r="M116" s="12" t="n"/>
       <c r="N116" s="12" t="n"/>
       <c r="O116" s="6" t="n"/>
+      <c r="P116" s="6" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="12">
@@ -3444,6 +3559,7 @@
       <c r="M117" s="12" t="n"/>
       <c r="N117" s="12" t="n"/>
       <c r="O117" s="6" t="n"/>
+      <c r="P117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="12">
@@ -3467,6 +3583,7 @@
       <c r="M118" s="12" t="n"/>
       <c r="N118" s="12" t="n"/>
       <c r="O118" s="6" t="n"/>
+      <c r="P118" s="6" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="12">
@@ -3490,6 +3607,7 @@
       <c r="M119" s="12" t="n"/>
       <c r="N119" s="12" t="n"/>
       <c r="O119" s="6" t="n"/>
+      <c r="P119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="12">
@@ -3513,6 +3631,7 @@
       <c r="M120" s="12" t="n"/>
       <c r="N120" s="12" t="n"/>
       <c r="O120" s="6" t="n"/>
+      <c r="P120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="12">
@@ -3536,6 +3655,7 @@
       <c r="M121" s="12" t="n"/>
       <c r="N121" s="12" t="n"/>
       <c r="O121" s="6" t="n"/>
+      <c r="P121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="12">
@@ -3559,6 +3679,7 @@
       <c r="M122" s="12" t="n"/>
       <c r="N122" s="12" t="n"/>
       <c r="O122" s="6" t="n"/>
+      <c r="P122" s="6" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="12">
@@ -3582,6 +3703,7 @@
       <c r="M123" s="12" t="n"/>
       <c r="N123" s="12" t="n"/>
       <c r="O123" s="6" t="n"/>
+      <c r="P123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="12">
@@ -3605,6 +3727,7 @@
       <c r="M124" s="12" t="n"/>
       <c r="N124" s="12" t="n"/>
       <c r="O124" s="6" t="n"/>
+      <c r="P124" s="6" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="12">
@@ -3628,6 +3751,7 @@
       <c r="M125" s="12" t="n"/>
       <c r="N125" s="12" t="n"/>
       <c r="O125" s="6" t="n"/>
+      <c r="P125" s="6" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="12">
@@ -3651,6 +3775,7 @@
       <c r="M126" s="12" t="n"/>
       <c r="N126" s="12" t="n"/>
       <c r="O126" s="6" t="n"/>
+      <c r="P126" s="6" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="12">
@@ -3674,6 +3799,7 @@
       <c r="M127" s="12" t="n"/>
       <c r="N127" s="12" t="n"/>
       <c r="O127" s="6" t="n"/>
+      <c r="P127" s="6" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="12">
@@ -3697,6 +3823,7 @@
       <c r="M128" s="12" t="n"/>
       <c r="N128" s="12" t="n"/>
       <c r="O128" s="6" t="n"/>
+      <c r="P128" s="6" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="12">
@@ -3720,18 +3847,19 @@
       <c r="M129" s="12" t="n"/>
       <c r="N129" s="12" t="n"/>
       <c r="O129" s="6" t="n"/>
+      <c r="P129" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A7:O7"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="C1:O1"/>
-    <mergeCell ref="C2:O2"/>
+    <mergeCell ref="C2:P2"/>
+    <mergeCell ref="A6:P6"/>
+    <mergeCell ref="C1:P1"/>
+    <mergeCell ref="A7:P7"/>
   </mergeCells>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Project / Client" prompt="Type the project name (new jobs welcome). It auto-fills down column A."/>
     <dataValidation sqref="G4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="MRA Job #" prompt="Job number if you have one, or type &quot;NEW&quot;."/>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Project Manager" prompt="The PM for this project — auto-fills down column J."/>
@@ -3754,6 +3882,7 @@
     <dataValidation sqref="O10:O129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$H$2:$H$2</formula1>
     </dataValidation>
+    <dataValidation sqref="P10:P129" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Sub-Resource" prompt="Optional — the person within the Assigned-To GROUP. e.g. Assigned To = &quot;MRA Design&quot;, Sub-Resource = &quot;Steve K&quot;. The dashboard rolls members up under their group, and lets you view just that person."/>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$F$2:$F$14</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Intake template: rename Post Production -> QA, add Warranty / Post-Launch Repairs phase
build_template.py Phase list updated + dropdown range extended to B11; regenerated
MRA_Project_Intake_Template.xlsx. Publishes on a mode=live deploy. (Al #14/#15.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJTcYohvXPdyiEYiaxvXwj
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -3865,7 +3865,7 @@
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Project Manager" prompt="The PM for this project — auto-fills down column J."/>
     <dataValidation sqref="D14 D15 D20 D21 D26 D27 D32 D33 D38 D39 D44 D45 D50 D51 D56 D57 D62 D63 D68 D69" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Subtask" prompt="Subtask of the task above. Type the subtask here and keep the &quot;x&quot; in the Sub column — the dashboard nests it (collapsible) under its parent. Clear the &quot;x&quot; to make it a normal task."/>
     <dataValidation sqref="B10:B129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$B$2:$B$10</formula1>
+      <formula1>=Lists!$B$2:$B$11</formula1>
     </dataValidation>
     <dataValidation sqref="C10:C129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$C$2:$C$10</formula1>
@@ -4132,7 +4132,7 @@
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Post Production</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4174,6 +4174,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Warranty / Post-Launch Repairs</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>Cindy Irland</t>

</xml_diff>

<commit_message>
Update MRA logo everywhere (rev 36.82)
Replaces logo.png with the current mark (adds the mobile.experiential
wordmark, transparent background instead of white) -- this file feeds
the dashboard header/favicon, every report letterhead, the Quote
Generator, and Design Team board. Also regenerated the Product
Catalogue's separately-embedded copy and the downloadable Project
Intake Template. Fixed two small icon spots (Design board napkin-mode
brand icon, Design Team Board header) that had fixed square dimensions
with no object-fit -- they'd have stretched the new, taller logo;
added object-fit:cover so they crop cleanly instead. Also fixed
build_template.py's hardcoded square image size to compute from the
logo's real aspect ratio so this doesn't break again next time the
logo changes.
</commit_message>
<xml_diff>
--- a/MRA_Project_Intake_Template.xlsx
+++ b/MRA_Project_Intake_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Enter Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lists" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enter Here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" state="veryHidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -234,20 +234,20 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="704850" cy="704850"/>
+    <ext cx="704850" cy="800100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>